<commit_message>
Pre Market Mon 2026-07-13
</commit_message>
<xml_diff>
--- a/market-prep/Pre Market 2026-07-13.xlsx
+++ b/market-prep/Pre Market 2026-07-13.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7579,53</t>
+          <t>7575,39</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29831,62</t>
+          <t>29825,11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52698,82</t>
+          <t>52637,01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4112,20</t>
+          <t>4120,38</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>59,77</t>
+          <t>59,83</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1632,40</t>
+          <t>1630,70</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>76,08</t>
+          <t>76,01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>63845,46</t>
+          <t>63943,89</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1790,61</t>
+          <t>1790,81</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-4,86%</t>
+          <t>-5,11%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7575,91</t>
+          <t>7575,39</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>

</xml_diff>